<commit_message>
feat(costes): enhance cost analysis and product export functionality
- Added a new function `exportar_coste_por_producto_excel` to generate detailed cost reports by product for specified periods, improving financial tracking.
- Updated the `analisis_costes.py` page to include options for downloading cost reports for the current week, month, and selected periods, enhancing user accessibility to financial data.
- Improved the presentation layer to display product costs and usage statistics, providing clearer insights into cost distribution.

This update significantly enhances the cost management features, allowing for better financial oversight and reporting capabilities.
</commit_message>
<xml_diff>
--- a/docs/plantillas/registro_desayuno_operativo_LISTA_ACTUALIZADA_ACTUALIZADA.xlsx
+++ b/docs/plantillas/registro_desayuno_operativo_LISTA_ACTUALIZADA_ACTUALIZADA.xlsx
@@ -503,6 +503,9 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -520,173 +523,223 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2. En cada línea ponga la Fecha (AAAA-MM-DD). Misma fecha = un solo desayuno en BM.</t>
+          <t>2. En cada línea ponga la Fecha (AAAA-MM-DD). Misma fecha = UN solo desayuno en BM.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3. Huespedes: basta en la primera línea de ese día (si vacío, se cuenta 1 por línea Receta).</t>
+          <t>3. Huéspedes (por línea, se SUMAN en el día):</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>4. Tipo: Receta (plato/bebida), Extra (buffet rápido) o Producto (mismo catálogo de extras).</t>
+          <t xml:space="preserve">   • 1 = nuevo comensal (cuenta 1 persona).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>5. Nombre: elija del desplegable (lista en hoja Catalogo).</t>
+          <t xml:space="preserve">   • 0 = mismo comensal que pide otro plato (NO suma persona).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>6. Cantidad ↑↓: raciones o unidades. Escriba un número 1–30.</t>
+          <t xml:space="preserve">   • Vacío = igual que 0 (no suma).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>7. Extra1…Extra4: extras sobre una Receta (bacon, aguacate, huevo, pan, etc.).</t>
+          <t xml:space="preserve">   Ejemplo: comensal pide inglés + café → fila inglés Huespedes=1, fila café=0.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8. Omitir1/Omitir2: quitar un ingrediente (Bacon, Sin huevo, Sin tostada…).</t>
+          <t xml:space="preserve">   Total del día = suma de la columna (solo los 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>4. Tipo: Receta (plato/bebida), Extra (buffet rápido) o Producto.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>HUEVOS (Desayuno inglés)</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>5. Nombre: elija del desplegable (lista en hoja Catalogo).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>• La ficha «Desayuno ingles» incluye Huevo frito por defecto.</t>
+          <t>6. Cantidad ↑↓: raciones o unidades de ESA línea (1–30).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>• Para otro tipo: Extra1 = Huevo pochado / Huevos revueltos / Huevo cocido</t>
+          <t>7. Extra1…Extra4: extras sobre una Receta (bacon, aguacate, huevo, pan…).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (sustituye al frito; no sume un segundo huevo).</t>
+          <t>8. Omitir1/Omitir2: quitar un ingrediente (Bacon, Sin huevo, Sin tostada…).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>• Para sin huevo: Omitir1 = Sin huevo (o Huevo frito).</t>
-        </is>
-      </c>
+      <c r="A17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>• Para huevo suelto (no inglés): Tipo=Receta y Nombre=Huevo frito / pochado / …</t>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>IMPORTANTE</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  o Tipo=Extra y Nombre=Huevo frito (añade al buffet).</t>
+          <t>• No ponga 1 en todas las filas: si lo hace, contará 1 huésped por plato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>• Cantidad es raciones del plato, no el número de huéspedes.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>PAN (tostadas / sándwiches)</t>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>• Tras importar, puede borrar las filas del Excel; en BM ya queda el registro.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>• Por defecto las fichas llevan molde común (blanco) = «Tostada» / «Pan blanco».</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>• Para integral: Extra1 = Tostada integral (o Pan integral).</t>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>HUEVOS (Desayuno inglés)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>• Para sin gluten: Extra1 = Tostada sin gluten (o Pan sin gluten)</t>
+          <t>• La ficha «Desayuno ingles» incluye Huevo frito por defecto.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  → panecillo s/gluten Betina; sustituye el pan de la ficha (1 reb → 1 ud).</t>
+          <t>• Para otro tipo: Extra1 = Huevo pochado / Huevos revueltos / Huevo cocido</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>• Para volver a blanco: Extra1 = Tostada / Pan blanco.</t>
+          <t xml:space="preserve">  (sustituye al frito; no sume un segundo huevo).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• Sin pan: Omitir1 = Sin tostada.</t>
+          <t>• Para sin huevo: Omitir1 = Sin huevo (o Huevo frito).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• Pan suelto de buffet: Tipo=Extra y Nombre=Tostada / integral / sin gluten.</t>
-        </is>
-      </c>
+          <t>• Huevo suelto: Tipo=Receta y Nombre=Huevo frito / pochado / …</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>9. Guarde el archivo y ejecute el importador (ver 2_importar_a_bm.cmd).</t>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>PAN (tostadas / sándwiches)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>10. Use --dry-run primero. La columna Importado la rellena el script.</t>
+          <t>• Por defecto: molde común (blanco) = Tostada / Pan blanco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>• Integral: Extra1 = Tostada integral (o Pan integral).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
+        <is>
+          <t>• Sin gluten: Extra1 = Tostada sin gluten (o Pan sin gluten).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>• Sin pan: Omitir1 = Sin tostada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>9. Guarde y ejecute 2_importar_a_bm.cmd (mejor --dry-run antes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>10. La columna Importado la rellena el script (no la edite).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>Al regenerar la plantilla NO se borran las filas ya rellenadas en Registro.</t>
         </is>
@@ -866,7 +919,7 @@
       <c r="P2" s="7" t="n"/>
       <c r="Q2" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -903,7 +956,7 @@
       <c r="P3" s="7" t="n"/>
       <c r="Q3" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -946,7 +999,7 @@
       <c r="P4" s="7" t="n"/>
       <c r="Q4" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -983,7 +1036,7 @@
       <c r="P5" s="7" t="n"/>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1079,7 @@
       <c r="P6" s="7" t="n"/>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1124,7 @@
       <c r="P7" s="7" t="n"/>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1161,7 @@
       <c r="P8" s="7" t="n"/>
       <c r="Q8" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1210,7 @@
       <c r="P9" s="7" t="n"/>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1257,7 @@
       <c r="P10" s="7" t="n"/>
       <c r="Q10" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1294,7 @@
       <c r="P11" s="7" t="n"/>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1331,7 @@
       <c r="P12" s="7" t="n"/>
       <c r="Q12" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1368,7 @@
       <c r="P13" s="7" t="n"/>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1405,7 @@
       <c r="P14" s="7" t="n"/>
       <c r="Q14" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1442,7 @@
       <c r="P15" s="7" t="n"/>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1479,7 @@
       <c r="P16" s="7" t="n"/>
       <c r="Q16" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1534,7 @@
       <c r="P17" s="7" t="n"/>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1577,7 @@
       <c r="P18" s="7" t="n"/>
       <c r="Q18" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1626,7 @@
       <c r="P19" s="7" t="n"/>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1673,7 @@
       <c r="P20" s="7" t="n"/>
       <c r="Q20" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1716,7 @@
       <c r="P21" s="7" t="n"/>
       <c r="Q21" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1777,7 @@
       <c r="P22" s="7" t="n"/>
       <c r="Q22" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1838,7 @@
       <c r="P23" s="7" t="n"/>
       <c r="Q23" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1887,7 @@
       <c r="P24" s="7" t="n"/>
       <c r="Q24" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1930,7 @@
       <c r="P25" s="7" t="n"/>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1938,7 +1991,7 @@
       <c r="P26" s="7" t="n"/>
       <c r="Q26" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -1981,7 +2034,7 @@
       <c r="P27" s="7" t="n"/>
       <c r="Q27" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2077,7 @@
       <c r="P28" s="7" t="n"/>
       <c r="Q28" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2114,7 @@
       <c r="P29" s="7" t="n"/>
       <c r="Q29" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2163,7 @@
       <c r="P30" s="7" t="n"/>
       <c r="Q30" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>
@@ -2159,7 +2212,7 @@
       <c r="P31" s="7" t="n"/>
       <c r="Q31" s="7" t="inlineStr">
         <is>
-          <t>OK d151, d152, d153, d154, d155, d156, d157, d158, d159, d160, d161, d162, d163, d164, d165, d166, d167, d168, d169, d170, d171, d172, d173, d174, d175, d176, d177, d178, d179, d180</t>
+          <t>OK d181</t>
         </is>
       </c>
     </row>

</xml_diff>